<commit_message>
paper run 2026-10-21 09:42
</commit_message>
<xml_diff>
--- a/reports/2026-10-21.xlsx
+++ b/reports/2026-10-21.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -472,6 +472,49 @@
         <is>
           <t>P&amp;L $</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-10-21T07:41:33.826918+00:00</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>15</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="F2" t="n">
+        <v>54.63</v>
+      </c>
+      <c r="G2" t="n">
+        <v>101.17</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.782</v>
+      </c>
+      <c r="I2" t="n">
+        <v>-0.00169</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
+        <v>46.54</v>
       </c>
     </row>
   </sheetData>
@@ -485,7 +528,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -507,7 +550,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -517,7 +560,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -536,6 +579,9 @@
           <t>winrate</t>
         </is>
       </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -544,7 +590,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>46.54</v>
       </c>
     </row>
     <row r="7">
@@ -554,7 +600,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>46.54</v>
       </c>
     </row>
     <row r="8">
@@ -573,6 +619,9 @@
           <t>pf</t>
         </is>
       </c>
+      <c r="B9" t="n">
+        <v>99</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -581,7 +630,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3585.559999999999</v>
+        <v>3632.099999999999</v>
       </c>
     </row>
     <row r="12">
@@ -628,161 +677,409 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" t="n">
+        <v>324.97</v>
+      </c>
+      <c r="E15" t="n">
+        <v>46.54</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="n">
+        <v>142.69</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>По активам</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" t="n">
+        <v>152.72</v>
+      </c>
+      <c r="E18" t="n">
+        <v>46.54</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" t="n">
+        <v>314.94</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>По цене входа</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>2</v>
+      </c>
+      <c r="C21" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" t="n">
+        <v>324.97</v>
+      </c>
+      <c r="E21" t="n">
+        <v>46.54</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" t="n">
+        <v>142.69</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>По окнам</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>По риск-гейтам</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>2</v>
+      </c>
+      <c r="C24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" t="n">
+        <v>314.94</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>По часам</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" t="n">
+        <v>152.72</v>
+      </c>
+      <c r="E25" t="n">
+        <v>46.54</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
+          <t>REALIZED (реальные сделки)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>По активам</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>1</v>
+      </c>
+      <c r="C30" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" t="n">
+        <v>46.54</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>По окнам</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>15m</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>1</v>
+      </c>
+      <c r="C33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" t="n">
+        <v>46.54</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>1</v>
+      </c>
+      <c r="C36" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" t="n">
+        <v>46.54</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>По цене входа</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" t="n">
+        <v>46.54</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>По силе движения</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>1</v>
+      </c>
+      <c r="C42" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" t="n">
+        <v>46.54</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
         <is>
           <t>По направлению</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B44" t="inlineStr">
         <is>
           <t>сделок</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>побед</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t>P&amp;L</t>
         </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" t="n">
+        <v>1</v>
+      </c>
+      <c r="D45" t="n">
+        <v>46.54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
paper run 2026-10-21 16:58
</commit_message>
<xml_diff>
--- a/reports/2026-10-21.xlsx
+++ b/reports/2026-10-21.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -515,6 +515,92 @@
       </c>
       <c r="K2" t="n">
         <v>46.54</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-10-21T12:41:15.944761+00:00</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="F3" t="n">
+        <v>5.27</v>
+      </c>
+      <c r="G3" t="n">
+        <v>9.949999999999999</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.757</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.00108</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>4.68</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-10-21T15:03:50.626881+00:00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>SOL</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>DOWN</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.6038</v>
+      </c>
+      <c r="F4" t="n">
+        <v>123.1</v>
+      </c>
+      <c r="G4" t="n">
+        <v>203.87</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.769</v>
+      </c>
+      <c r="I4" t="n">
+        <v>-0.0013</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
+        <v>80.77</v>
       </c>
     </row>
   </sheetData>
@@ -528,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -550,7 +636,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -560,7 +646,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -590,7 +676,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>46.54</v>
+        <v>131.99</v>
       </c>
     </row>
     <row r="7">
@@ -600,7 +686,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>46.54</v>
+        <v>131.99</v>
       </c>
     </row>
     <row r="8">
@@ -630,7 +716,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>3632.099999999999</v>
+        <v>3717.549999999999</v>
       </c>
     </row>
     <row r="12">
@@ -681,16 +767,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D15" t="n">
-        <v>324.97</v>
+        <v>1009.53</v>
       </c>
       <c r="E15" t="n">
-        <v>46.54</v>
+        <v>51.22</v>
       </c>
     </row>
     <row r="16">
@@ -700,16 +786,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D16" t="n">
-        <v>142.69</v>
+        <v>563.89</v>
       </c>
       <c r="E16" t="n">
-        <v>0</v>
+        <v>80.77</v>
       </c>
     </row>
     <row r="17">
@@ -722,7 +808,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SOL</t>
+          <t>ETH</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -732,170 +818,189 @@
         <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>152.72</v>
+        <v>150.43</v>
       </c>
       <c r="E18" t="n">
-        <v>46.54</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>XRP</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C19" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D19" t="n">
-        <v>314.94</v>
+        <v>587.6</v>
       </c>
       <c r="E19" t="n">
-        <v>0</v>
+        <v>131.99</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>По цене входа</t>
-        </is>
+          <t>XRP</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>6</v>
+      </c>
+      <c r="C20" t="n">
+        <v>6</v>
+      </c>
+      <c r="D20" t="n">
+        <v>835.39</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>2</v>
-      </c>
-      <c r="C21" t="n">
-        <v>2</v>
-      </c>
-      <c r="D21" t="n">
-        <v>324.97</v>
-      </c>
-      <c r="E21" t="n">
-        <v>46.54</v>
+          <t>По цене входа</t>
+        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0.55–0.60</t>
+          <t>0.50–0.55</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D22" t="n">
-        <v>142.69</v>
+        <v>1136.75</v>
       </c>
       <c r="E22" t="n">
-        <v>0</v>
+        <v>51.22</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>По риск-гейтам</t>
-        </is>
+          <t>0.55–0.60</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1</v>
+      </c>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" t="n">
+        <v>142.69</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>NO_LIQUIDITY</t>
+          <t>0.60–0.62</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D24" t="n">
-        <v>314.94</v>
+        <v>293.98</v>
       </c>
       <c r="E24" t="n">
-        <v>0</v>
+        <v>80.77</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>1</v>
-      </c>
-      <c r="C25" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" t="n">
-        <v>152.72</v>
-      </c>
-      <c r="E25" t="n">
-        <v>46.54</v>
+          <t>По риск-гейтам</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>MAX_PER_WINDOW</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" t="n">
+        <v>150.43</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>REALIZED (реальные сделки)</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>По активам</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>NO_LIQUIDITY</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>7</v>
+      </c>
+      <c r="C27" t="n">
+        <v>7</v>
+      </c>
+      <c r="D27" t="n">
+        <v>1017.23</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>3</v>
+      </c>
+      <c r="C28" t="n">
+        <v>3</v>
+      </c>
+      <c r="D28" t="n">
+        <v>405.76</v>
+      </c>
+      <c r="E28" t="n">
+        <v>131.99</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SOL</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>1</v>
-      </c>
-      <c r="C30" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" t="n">
-        <v>46.54</v>
+          <t>REALIZED (реальные сделки)</t>
+        </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>По окнам</t>
+          <t>По активам</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -917,23 +1022,23 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>15m</t>
+          <t>SOL</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C33" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D33" t="n">
-        <v>46.54</v>
+        <v>131.99</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>По часам</t>
+          <t>По окнам</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -955,83 +1060,93 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>07</t>
+          <t>15m</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D36" t="n">
-        <v>46.54</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>По цене входа</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+        <v>51.22</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>5m</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" t="n">
+        <v>80.77</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>0.50–0.55</t>
-        </is>
-      </c>
-      <c r="B39" t="n">
-        <v>1</v>
-      </c>
-      <c r="C39" t="n">
-        <v>1</v>
-      </c>
-      <c r="D39" t="n">
+          <t>По часам</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>07</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>1</v>
+      </c>
+      <c r="C40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" t="n">
         <v>46.54</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>По силе движения</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>сделок</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>побед</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>P&amp;L</t>
-        </is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" t="n">
+        <v>4.68</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>0.15–0.20%</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1041,13 +1156,13 @@
         <v>1</v>
       </c>
       <c r="D42" t="n">
-        <v>46.54</v>
+        <v>80.77</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>По направлению</t>
+          <t>По цене входа</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1069,17 +1184,157 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>0.50–0.55</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>2</v>
+      </c>
+      <c r="C45" t="n">
+        <v>2</v>
+      </c>
+      <c r="D45" t="n">
+        <v>51.22</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>0.60–0.62</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" t="n">
+        <v>80.77</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>По силе движения</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>0.10–0.12%</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>1</v>
+      </c>
+      <c r="C49" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" t="n">
+        <v>4.68</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>0.12–0.15%</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>1</v>
+      </c>
+      <c r="C50" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" t="n">
+        <v>80.77</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>0.15–0.20%</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>1</v>
+      </c>
+      <c r="C51" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" t="n">
+        <v>46.54</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>По направлению</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>сделок</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>побед</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>P&amp;L</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
           <t>DOWN</t>
         </is>
       </c>
-      <c r="B45" t="n">
-        <v>1</v>
-      </c>
-      <c r="C45" t="n">
-        <v>1</v>
-      </c>
-      <c r="D45" t="n">
-        <v>46.54</v>
+      <c r="B54" t="n">
+        <v>2</v>
+      </c>
+      <c r="C54" t="n">
+        <v>2</v>
+      </c>
+      <c r="D54" t="n">
+        <v>127.31</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>UP</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>1</v>
+      </c>
+      <c r="C55" t="n">
+        <v>1</v>
+      </c>
+      <c r="D55" t="n">
+        <v>4.68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
paper run 2026-10-21 22:38
</commit_message>
<xml_diff>
--- a/reports/2026-10-21.xlsx
+++ b/reports/2026-10-21.xlsx
@@ -767,13 +767,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C15" t="n">
         <v>7</v>
       </c>
       <c r="D15" t="n">
-        <v>1009.53</v>
+        <v>823.65</v>
       </c>
       <c r="E15" t="n">
         <v>51.22</v>
@@ -850,13 +850,13 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C20" t="n">
         <v>6</v>
       </c>
       <c r="D20" t="n">
-        <v>835.39</v>
+        <v>649.51</v>
       </c>
       <c r="E20" t="n">
         <v>0</v>
@@ -876,13 +876,13 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C22" t="n">
         <v>7</v>
       </c>
       <c r="D22" t="n">
-        <v>1136.75</v>
+        <v>950.87</v>
       </c>
       <c r="E22" t="n">
         <v>51.22</v>
@@ -959,13 +959,13 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C27" t="n">
         <v>7</v>
       </c>
       <c r="D27" t="n">
-        <v>1017.23</v>
+        <v>831.35</v>
       </c>
       <c r="E27" t="n">
         <v>0</v>

</xml_diff>